<commit_message>
Organize project images and structure
</commit_message>
<xml_diff>
--- a/outputs/evaluation_results.xlsx
+++ b/outputs/evaluation_results.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>83.33%</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Evidence should identify the following for sustainability metrics:
+          <t>According to the Sustainability Reporting Guidelines, evidence should identify the following for sustainability metrics:
 1. Reporting period
 2. Measurement method
 3. Responsible department
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>

</xml_diff>